<commit_message>
chore(scripts): titulo en Configuracion Niveles.xlsx
Solo presentacion: se agrega el titulo "CONFIGURACION DE CUENTA CONTABLE" y
los datos bajan una fila. La tabla es la misma.

Es la referencia de la estructura del codigo de cuenta: segmentacion
{1,1,1,3,2,2} por nivel y su mapeo a cn_nivel, que implementa la validacion
del alta en CashAccountAction.analyzeAccountCode().

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/scripts/Configuracion Niveles.xlsx
+++ b/scripts/Configuracion Niveles.xlsx
@@ -5,12 +5,12 @@
   <workbookPr codeName="ThisWorkbook" defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Intellij\sisk13\view\plan_ctas\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Intellij\sisk13\scripts\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{547B1F7B-7A74-4DAF-A983-5BFBD096139D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B9E49FAC-3615-4F52-ADAE-115714969BB6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="8340" yWindow="1950" windowWidth="20115" windowHeight="12840" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="6780" windowWidth="13425" windowHeight="14805" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Hoja1" sheetId="2" r:id="rId1"/>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="44" uniqueCount="20">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="33" uniqueCount="20">
   <si>
     <t>cn_nivel</t>
   </si>
@@ -61,9 +61,6 @@
     <t>00</t>
   </si>
   <si>
-    <t>x</t>
-  </si>
-  <si>
     <t>1</t>
   </si>
   <si>
@@ -80,13 +77,16 @@
   </si>
   <si>
     <t>6</t>
+  </si>
+  <si>
+    <t>CONFIGURACION DE CUENTA CONTABLE</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="22" x14ac:knownFonts="1">
+  <fonts count="23" x14ac:knownFonts="1">
     <font>
       <sz val="10"/>
       <name val="Arial"/>
@@ -237,12 +237,17 @@
     <font>
       <b/>
       <sz val="14"/>
-      <color indexed="12"/>
+      <name val="Arial"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="14"/>
       <name val="Arial Narrow"/>
       <family val="2"/>
     </font>
   </fonts>
-  <fills count="34">
+  <fills count="36">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -424,12 +429,24 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor theme="0" tint="-4.9989318521683403E-2"/>
+        <fgColor theme="2" tint="-9.9978637043366805E-2"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="6" tint="0.79998168889431442"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="4" tint="0.79998168889431442"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
   </fills>
-  <borders count="10">
+  <borders count="11">
     <border>
       <left/>
       <right/>
@@ -544,6 +561,21 @@
       </bottom>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="42">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
@@ -589,7 +621,7 @@
     <xf numFmtId="0" fontId="1" fillId="31" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="1" fillId="32" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="10">
+  <cellXfs count="16">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="49" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
@@ -607,14 +639,30 @@
     <xf numFmtId="0" fontId="18" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf numFmtId="0" fontId="18" fillId="33" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="18" fillId="33" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="21" fillId="33" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="22" fillId="35" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="18" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="49" fontId="18" fillId="0" borderId="10" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="49" fontId="18" fillId="35" borderId="10" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="34" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="49" fontId="21" fillId="34" borderId="10" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="19" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center"/>
+      <alignment horizontal="left"/>
     </xf>
   </cellXfs>
   <cellStyles count="42">
@@ -981,186 +1029,183 @@
     <col min="9" max="9" width="11.42578125" style="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:8" ht="18" x14ac:dyDescent="0.25">
-      <c r="A1" s="9" t="s">
-        <v>4</v>
-      </c>
-      <c r="E1" s="5"/>
-      <c r="F1" s="5"/>
-      <c r="G1" s="5"/>
-      <c r="H1" s="5"/>
+    <row r="1" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="A1" s="14" t="s">
+        <v>19</v>
+      </c>
     </row>
     <row r="2" spans="1:8" ht="18" x14ac:dyDescent="0.25">
-      <c r="A2" s="6">
-        <v>1110040103</v>
-      </c>
-      <c r="B2" s="7" t="s">
-        <v>5</v>
-      </c>
-      <c r="C2" s="7" t="s">
-        <v>6</v>
-      </c>
-      <c r="D2" s="7" t="s">
-        <v>7</v>
-      </c>
-      <c r="E2" s="7" t="s">
-        <v>8</v>
-      </c>
-      <c r="F2" s="7" t="s">
-        <v>9</v>
-      </c>
-      <c r="G2" s="7" t="s">
-        <v>10</v>
-      </c>
-      <c r="H2" s="8" t="s">
-        <v>0</v>
-      </c>
+      <c r="A2" s="15" t="s">
+        <v>4</v>
+      </c>
+      <c r="E2" s="5"/>
+      <c r="F2" s="5"/>
+      <c r="G2" s="5"/>
+      <c r="H2" s="5"/>
     </row>
     <row r="3" spans="1:8" ht="18" x14ac:dyDescent="0.25">
-      <c r="B3" s="4">
-        <v>1</v>
-      </c>
-      <c r="C3" s="4">
+      <c r="A3" s="6">
+        <v>1110040103</v>
+      </c>
+      <c r="B3" s="7" t="s">
+        <v>5</v>
+      </c>
+      <c r="C3" s="7" t="s">
+        <v>6</v>
+      </c>
+      <c r="D3" s="7" t="s">
+        <v>7</v>
+      </c>
+      <c r="E3" s="7" t="s">
+        <v>8</v>
+      </c>
+      <c r="F3" s="7" t="s">
+        <v>9</v>
+      </c>
+      <c r="G3" s="7" t="s">
+        <v>10</v>
+      </c>
+      <c r="H3" s="8" t="s">
         <v>0</v>
-      </c>
-      <c r="D3" s="4">
-        <v>0</v>
-      </c>
-      <c r="E3" s="5" t="s">
-        <v>11</v>
-      </c>
-      <c r="F3" s="5" t="s">
-        <v>12</v>
-      </c>
-      <c r="G3" s="5" t="s">
-        <v>12</v>
-      </c>
-      <c r="H3" s="5" t="s">
-        <v>14</v>
       </c>
     </row>
     <row r="4" spans="1:8" ht="18" x14ac:dyDescent="0.25">
-      <c r="B4" s="4" t="s">
+      <c r="B4" s="9">
+        <v>1</v>
+      </c>
+      <c r="C4" s="9">
+        <v>0</v>
+      </c>
+      <c r="D4" s="9">
+        <v>0</v>
+      </c>
+      <c r="E4" s="10" t="s">
+        <v>11</v>
+      </c>
+      <c r="F4" s="10" t="s">
+        <v>12</v>
+      </c>
+      <c r="G4" s="10" t="s">
+        <v>12</v>
+      </c>
+      <c r="H4" s="11" t="s">
         <v>13</v>
-      </c>
-      <c r="C4" s="4">
-        <v>1</v>
-      </c>
-      <c r="D4" s="4">
-        <v>0</v>
-      </c>
-      <c r="E4" s="5" t="s">
-        <v>11</v>
-      </c>
-      <c r="F4" s="5" t="s">
-        <v>12</v>
-      </c>
-      <c r="G4" s="5" t="s">
-        <v>12</v>
-      </c>
-      <c r="H4" s="5" t="s">
-        <v>16</v>
       </c>
     </row>
     <row r="5" spans="1:8" ht="18" x14ac:dyDescent="0.25">
-      <c r="B5" s="4" t="s">
-        <v>13</v>
-      </c>
-      <c r="C5" s="4" t="s">
-        <v>13</v>
-      </c>
-      <c r="D5" s="4">
-        <v>1</v>
-      </c>
-      <c r="E5" s="5" t="s">
+      <c r="B5" s="9">
+        <v>1</v>
+      </c>
+      <c r="C5" s="9">
+        <v>1</v>
+      </c>
+      <c r="D5" s="9">
+        <v>0</v>
+      </c>
+      <c r="E5" s="10" t="s">
         <v>11</v>
       </c>
-      <c r="F5" s="5" t="s">
+      <c r="F5" s="10" t="s">
         <v>12</v>
       </c>
-      <c r="G5" s="5" t="s">
+      <c r="G5" s="10" t="s">
         <v>12</v>
       </c>
-      <c r="H5" s="5" t="s">
+      <c r="H5" s="11" t="s">
         <v>15</v>
       </c>
     </row>
     <row r="6" spans="1:8" ht="18" x14ac:dyDescent="0.25">
-      <c r="B6" s="4" t="s">
-        <v>13</v>
-      </c>
-      <c r="C6" s="4" t="s">
-        <v>13</v>
-      </c>
-      <c r="D6" s="4" t="s">
-        <v>13</v>
-      </c>
-      <c r="E6" s="5" t="s">
-        <v>1</v>
-      </c>
-      <c r="F6" s="5" t="s">
+      <c r="B6" s="9">
+        <v>1</v>
+      </c>
+      <c r="C6" s="9">
+        <v>1</v>
+      </c>
+      <c r="D6" s="9">
+        <v>1</v>
+      </c>
+      <c r="E6" s="10" t="s">
+        <v>11</v>
+      </c>
+      <c r="F6" s="10" t="s">
         <v>12</v>
       </c>
-      <c r="G6" s="5" t="s">
+      <c r="G6" s="10" t="s">
         <v>12</v>
       </c>
-      <c r="H6" s="5" t="s">
-        <v>17</v>
+      <c r="H6" s="11" t="s">
+        <v>14</v>
       </c>
     </row>
     <row r="7" spans="1:8" ht="18" x14ac:dyDescent="0.25">
-      <c r="B7" s="4" t="s">
-        <v>13</v>
-      </c>
-      <c r="C7" s="4" t="s">
-        <v>13</v>
-      </c>
-      <c r="D7" s="4" t="s">
-        <v>13</v>
-      </c>
-      <c r="E7" s="5" t="s">
-        <v>13</v>
-      </c>
-      <c r="F7" s="5" t="s">
-        <v>2</v>
-      </c>
-      <c r="G7" s="5" t="s">
+      <c r="B7" s="9">
+        <v>1</v>
+      </c>
+      <c r="C7" s="9">
+        <v>1</v>
+      </c>
+      <c r="D7" s="9">
+        <v>1</v>
+      </c>
+      <c r="E7" s="10" t="s">
+        <v>1</v>
+      </c>
+      <c r="F7" s="10" t="s">
         <v>12</v>
       </c>
-      <c r="H7" s="5" t="s">
-        <v>18</v>
+      <c r="G7" s="10" t="s">
+        <v>12</v>
+      </c>
+      <c r="H7" s="11" t="s">
+        <v>16</v>
       </c>
     </row>
     <row r="8" spans="1:8" ht="18" x14ac:dyDescent="0.25">
-      <c r="B8" s="4" t="s">
-        <v>13</v>
-      </c>
-      <c r="C8" s="4" t="s">
-        <v>13</v>
-      </c>
-      <c r="D8" s="4" t="s">
-        <v>13</v>
-      </c>
-      <c r="E8" s="5" t="s">
-        <v>13</v>
-      </c>
-      <c r="F8" s="5" t="s">
-        <v>13</v>
-      </c>
-      <c r="G8" s="5" t="s">
-        <v>3</v>
-      </c>
-      <c r="H8" s="5" t="s">
-        <v>19</v>
+      <c r="B8" s="9">
+        <v>1</v>
+      </c>
+      <c r="C8" s="9">
+        <v>1</v>
+      </c>
+      <c r="D8" s="9">
+        <v>1</v>
+      </c>
+      <c r="E8" s="10" t="s">
+        <v>1</v>
+      </c>
+      <c r="F8" s="10" t="s">
+        <v>2</v>
+      </c>
+      <c r="G8" s="10" t="s">
+        <v>12</v>
+      </c>
+      <c r="H8" s="11" t="s">
+        <v>17</v>
       </c>
     </row>
     <row r="9" spans="1:8" ht="18" x14ac:dyDescent="0.25">
-      <c r="B9" s="4"/>
-      <c r="C9" s="4"/>
-      <c r="D9" s="4"/>
-      <c r="E9" s="5"/>
-      <c r="F9" s="5"/>
-      <c r="G9" s="5"/>
+      <c r="B9" s="12">
+        <v>1</v>
+      </c>
+      <c r="C9" s="12">
+        <v>1</v>
+      </c>
+      <c r="D9" s="12">
+        <v>1</v>
+      </c>
+      <c r="E9" s="13" t="s">
+        <v>1</v>
+      </c>
+      <c r="F9" s="13" t="s">
+        <v>2</v>
+      </c>
+      <c r="G9" s="13" t="s">
+        <v>3</v>
+      </c>
+      <c r="H9" s="11" t="s">
+        <v>18</v>
+      </c>
     </row>
     <row r="11" spans="1:8" ht="18" x14ac:dyDescent="0.25">
       <c r="B11" s="4"/>

</xml_diff>